<commit_message>
Opzet andere invoer Excel. Maar nog geen consensus
</commit_message>
<xml_diff>
--- a/geoprob_pipe/pre_processing/parameter_input/parameter_input_template.xlsx
+++ b/geoprob_pipe/pre_processing/parameter_input/parameter_input_template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CP\git_clones\GeoProb-Pipe\GeoProb-PipeV2\GeoProb-Pipe\geoprob_pipe\pre_processing\parameter_input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E88C1B1C-E052-4727-8C1D-9AB56469090E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1ED80BED-1F52-47BD-B087-05C5A6E3F2A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4072986C-855A-4E04-BDA4-92C994E74780}"/>
   </bookViews>
@@ -715,17 +715,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DAEDF215-1BC2-44F5-8521-4305F21BD459}">
   <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.33203125" style="14" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="60.5546875" style="14" customWidth="1"/>
-    <col min="3" max="3" width="52.6640625" style="14" customWidth="1"/>
-    <col min="4" max="4" width="25.109375" style="14" customWidth="1"/>
-    <col min="5" max="5" width="26.44140625" style="14" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="8.88671875" style="14"/>
+    <col min="1" max="1" width="23.28515625" style="14" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="60.5703125" style="14" customWidth="1"/>
+    <col min="3" max="3" width="52.7109375" style="14" customWidth="1"/>
+    <col min="4" max="4" width="25.140625" style="14" customWidth="1"/>
+    <col min="5" max="5" width="26.42578125" style="14" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="8.85546875" style="14"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>12</v>
       </c>
@@ -742,14 +742,14 @@
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="13"/>
       <c r="B2" s="13"/>
       <c r="C2" s="13"/>
       <c r="D2" s="13"/>
       <c r="E2" s="13"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
         <v>9</v>
       </c>
@@ -766,7 +766,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="15" t="s">
         <v>0</v>
       </c>
@@ -797,15 +797,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9313D639-575E-4463-A991-9636CAC84E2D}">
   <dimension ref="A1:C21"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13" style="2" customWidth="1"/>
-    <col min="2" max="2" width="20" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12" style="2" customWidth="1"/>
-    <col min="4" max="16384" width="8.88671875" style="2"/>
+    <col min="1" max="1" width="13.28515625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="45.5703125" style="2" customWidth="1"/>
+    <col min="3" max="3" width="13" style="2" customWidth="1"/>
+    <col min="4" max="16384" width="8.85546875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
@@ -816,7 +816,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>8</v>
       </c>
@@ -827,7 +827,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:3" s="6" customFormat="1" ht="12" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" s="6" customFormat="1" ht="12" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>2</v>
       </c>
@@ -838,58 +838,58 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C4" s="7"/>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C5" s="7"/>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C6" s="7"/>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C7" s="7"/>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C8" s="7"/>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C9" s="7"/>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C10" s="7"/>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C11" s="7"/>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C12" s="7"/>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C13" s="7"/>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C14" s="7"/>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C15" s="7"/>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C16" s="7"/>
     </row>
-    <row r="17" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C17" s="7"/>
     </row>
-    <row r="18" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C18" s="7"/>
     </row>
-    <row r="19" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C19" s="7"/>
     </row>
-    <row r="20" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C20" s="7"/>
     </row>
-    <row r="21" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C21" s="7"/>
     </row>
   </sheetData>
@@ -901,21 +901,21 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E90D4119-5ABA-4602-81BD-BF6C31F178E4}">
   <dimension ref="A1:J4"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="22.88671875" style="11" customWidth="1"/>
+    <col min="1" max="2" width="22.85546875" style="11" customWidth="1"/>
     <col min="3" max="3" width="13" style="11" customWidth="1"/>
-    <col min="4" max="4" width="26.5546875" style="11" customWidth="1"/>
-    <col min="5" max="5" width="15.33203125" style="11" customWidth="1"/>
-    <col min="6" max="6" width="21.5546875" style="11" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.88671875" style="11" customWidth="1"/>
-    <col min="8" max="8" width="12.33203125" style="11" customWidth="1"/>
-    <col min="9" max="9" width="38.88671875" style="11" customWidth="1"/>
+    <col min="4" max="4" width="26.5703125" style="11" customWidth="1"/>
+    <col min="5" max="5" width="15.28515625" style="11" customWidth="1"/>
+    <col min="6" max="6" width="21.5703125" style="11" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.85546875" style="11" customWidth="1"/>
+    <col min="8" max="8" width="12.28515625" style="11" customWidth="1"/>
+    <col min="9" max="9" width="38.85546875" style="11" customWidth="1"/>
     <col min="10" max="10" width="66" style="11" customWidth="1"/>
-    <col min="11" max="16384" width="8.88671875" style="11"/>
+    <col min="11" max="16384" width="8.85546875" style="11"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>12</v>
       </c>
@@ -945,7 +945,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="126.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" ht="126.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="16" t="s">
         <v>38</v>
       </c>
@@ -975,7 +975,7 @@
       </c>
       <c r="J2" s="16"/>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>9</v>
       </c>
@@ -1007,7 +1007,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>0</v>
       </c>
@@ -1048,18 +1048,18 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BEE6525A-680B-4461-9F3B-3E1CE43163B1}">
   <dimension ref="A1:G21"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13" style="2" customWidth="1"/>
-    <col min="2" max="2" width="72.44140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="44.109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.88671875" style="2"/>
-    <col min="5" max="6" width="10.6640625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="72.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="44.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.85546875" style="2"/>
+    <col min="5" max="6" width="10.7109375" style="2" customWidth="1"/>
     <col min="7" max="7" width="35" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="8.88671875" style="2"/>
+    <col min="8" max="16384" width="8.85546875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
         <v>43</v>
       </c>
@@ -1082,7 +1082,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="48" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A2" s="19" t="s">
         <v>47</v>
       </c>
@@ -1097,7 +1097,7 @@
       </c>
       <c r="G2" s="18"/>
     </row>
-    <row r="3" spans="1:7" s="6" customFormat="1" ht="12" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" s="6" customFormat="1" ht="12" x14ac:dyDescent="0.25">
       <c r="A3" s="18" t="s">
         <v>46</v>
       </c>
@@ -1120,59 +1120,59 @@
         <v>59</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C4" s="7"/>
       <c r="G4" s="7"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C5" s="7"/>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C6" s="7"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C7" s="7"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C8" s="7"/>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C9" s="7"/>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C10" s="7"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C11" s="7"/>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C12" s="7"/>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C13" s="7"/>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C14" s="7"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C15" s="7"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C16" s="7"/>
     </row>
-    <row r="17" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C17" s="7"/>
     </row>
-    <row r="18" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C18" s="7"/>
     </row>
-    <row r="19" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C19" s="7"/>
     </row>
-    <row r="20" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C20" s="7"/>
     </row>
-    <row r="21" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C21" s="7"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Verbeteringen n.a.v. beoordeling dijktraject 38-2 (#29)
* Tussenstand

* Fixed bug: anticipating no result in vak

* Small additions made to pre-processing

* Busy with point clicking algorithm

* First uittredepunten algo toegevoegd

* kleine aanpassing

* Small bug fix

* Opzet andere invoer Excel. Maar nog geen consensus

* some small changes

* Small change
</commit_message>
<xml_diff>
--- a/geoprob_pipe/pre_processing/parameter_input/parameter_input_template.xlsx
+++ b/geoprob_pipe/pre_processing/parameter_input/parameter_input_template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CP\git_clones\GeoProb-Pipe\GeoProb-PipeV2\GeoProb-Pipe\geoprob_pipe\pre_processing\parameter_input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E88C1B1C-E052-4727-8C1D-9AB56469090E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1ED80BED-1F52-47BD-B087-05C5A6E3F2A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4072986C-855A-4E04-BDA4-92C994E74780}"/>
   </bookViews>
@@ -715,17 +715,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DAEDF215-1BC2-44F5-8521-4305F21BD459}">
   <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.33203125" style="14" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="60.5546875" style="14" customWidth="1"/>
-    <col min="3" max="3" width="52.6640625" style="14" customWidth="1"/>
-    <col min="4" max="4" width="25.109375" style="14" customWidth="1"/>
-    <col min="5" max="5" width="26.44140625" style="14" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="8.88671875" style="14"/>
+    <col min="1" max="1" width="23.28515625" style="14" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="60.5703125" style="14" customWidth="1"/>
+    <col min="3" max="3" width="52.7109375" style="14" customWidth="1"/>
+    <col min="4" max="4" width="25.140625" style="14" customWidth="1"/>
+    <col min="5" max="5" width="26.42578125" style="14" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="8.85546875" style="14"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>12</v>
       </c>
@@ -742,14 +742,14 @@
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="13"/>
       <c r="B2" s="13"/>
       <c r="C2" s="13"/>
       <c r="D2" s="13"/>
       <c r="E2" s="13"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
         <v>9</v>
       </c>
@@ -766,7 +766,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="15" t="s">
         <v>0</v>
       </c>
@@ -797,15 +797,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9313D639-575E-4463-A991-9636CAC84E2D}">
   <dimension ref="A1:C21"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13" style="2" customWidth="1"/>
-    <col min="2" max="2" width="20" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12" style="2" customWidth="1"/>
-    <col min="4" max="16384" width="8.88671875" style="2"/>
+    <col min="1" max="1" width="13.28515625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="45.5703125" style="2" customWidth="1"/>
+    <col min="3" max="3" width="13" style="2" customWidth="1"/>
+    <col min="4" max="16384" width="8.85546875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
@@ -816,7 +816,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>8</v>
       </c>
@@ -827,7 +827,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:3" s="6" customFormat="1" ht="12" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" s="6" customFormat="1" ht="12" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>2</v>
       </c>
@@ -838,58 +838,58 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C4" s="7"/>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C5" s="7"/>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C6" s="7"/>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C7" s="7"/>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C8" s="7"/>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C9" s="7"/>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C10" s="7"/>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C11" s="7"/>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C12" s="7"/>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C13" s="7"/>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C14" s="7"/>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C15" s="7"/>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C16" s="7"/>
     </row>
-    <row r="17" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C17" s="7"/>
     </row>
-    <row r="18" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C18" s="7"/>
     </row>
-    <row r="19" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C19" s="7"/>
     </row>
-    <row r="20" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C20" s="7"/>
     </row>
-    <row r="21" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C21" s="7"/>
     </row>
   </sheetData>
@@ -901,21 +901,21 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E90D4119-5ABA-4602-81BD-BF6C31F178E4}">
   <dimension ref="A1:J4"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="22.88671875" style="11" customWidth="1"/>
+    <col min="1" max="2" width="22.85546875" style="11" customWidth="1"/>
     <col min="3" max="3" width="13" style="11" customWidth="1"/>
-    <col min="4" max="4" width="26.5546875" style="11" customWidth="1"/>
-    <col min="5" max="5" width="15.33203125" style="11" customWidth="1"/>
-    <col min="6" max="6" width="21.5546875" style="11" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.88671875" style="11" customWidth="1"/>
-    <col min="8" max="8" width="12.33203125" style="11" customWidth="1"/>
-    <col min="9" max="9" width="38.88671875" style="11" customWidth="1"/>
+    <col min="4" max="4" width="26.5703125" style="11" customWidth="1"/>
+    <col min="5" max="5" width="15.28515625" style="11" customWidth="1"/>
+    <col min="6" max="6" width="21.5703125" style="11" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.85546875" style="11" customWidth="1"/>
+    <col min="8" max="8" width="12.28515625" style="11" customWidth="1"/>
+    <col min="9" max="9" width="38.85546875" style="11" customWidth="1"/>
     <col min="10" max="10" width="66" style="11" customWidth="1"/>
-    <col min="11" max="16384" width="8.88671875" style="11"/>
+    <col min="11" max="16384" width="8.85546875" style="11"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>12</v>
       </c>
@@ -945,7 +945,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="126.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" ht="126.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="16" t="s">
         <v>38</v>
       </c>
@@ -975,7 +975,7 @@
       </c>
       <c r="J2" s="16"/>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>9</v>
       </c>
@@ -1007,7 +1007,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>0</v>
       </c>
@@ -1048,18 +1048,18 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BEE6525A-680B-4461-9F3B-3E1CE43163B1}">
   <dimension ref="A1:G21"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13" style="2" customWidth="1"/>
-    <col min="2" max="2" width="72.44140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="44.109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.88671875" style="2"/>
-    <col min="5" max="6" width="10.6640625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="72.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="44.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.85546875" style="2"/>
+    <col min="5" max="6" width="10.7109375" style="2" customWidth="1"/>
     <col min="7" max="7" width="35" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="8.88671875" style="2"/>
+    <col min="8" max="16384" width="8.85546875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
         <v>43</v>
       </c>
@@ -1082,7 +1082,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="48" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A2" s="19" t="s">
         <v>47</v>
       </c>
@@ -1097,7 +1097,7 @@
       </c>
       <c r="G2" s="18"/>
     </row>
-    <row r="3" spans="1:7" s="6" customFormat="1" ht="12" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" s="6" customFormat="1" ht="12" x14ac:dyDescent="0.25">
       <c r="A3" s="18" t="s">
         <v>46</v>
       </c>
@@ -1120,59 +1120,59 @@
         <v>59</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C4" s="7"/>
       <c r="G4" s="7"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C5" s="7"/>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C6" s="7"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C7" s="7"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C8" s="7"/>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C9" s="7"/>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C10" s="7"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C11" s="7"/>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C12" s="7"/>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C13" s="7"/>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C14" s="7"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C15" s="7"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C16" s="7"/>
     </row>
-    <row r="17" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C17" s="7"/>
     </row>
-    <row r="18" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C18" s="7"/>
     </row>
-    <row r="19" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C19" s="7"/>
     </row>
-    <row r="20" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C20" s="7"/>
     </row>
-    <row r="21" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C21" s="7"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Vaknaam toegevoegd aan export input excels
</commit_message>
<xml_diff>
--- a/geoprob_pipe/pre_processing/parameter_input/parameter_input_template.xlsx
+++ b/geoprob_pipe/pre_processing/parameter_input/parameter_input_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CP\git_clones\GeoProb-Pipe\GeoProb-PipeV2\GeoProb-Pipe\geoprob_pipe\pre_processing\parameter_input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05CDCA1E-A17C-485A-9941-7297465E50A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BD450CE-CDCB-41F7-AEF9-46B581B15214}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{4072986C-855A-4E04-BDA4-92C994E74780}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{4072986C-855A-4E04-BDA4-92C994E74780}"/>
   </bookViews>
   <sheets>
     <sheet name="Geohydrologisch model" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Geohydrologisch model'!$A$6:$E$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Parameter invoer'!$A$4:$H$336</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Scenario invoer'!$A$3:$C$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Scenario invoer'!$A$3:$D$3</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="72">
   <si>
     <t>parameter</t>
   </si>
@@ -110,9 +110,6 @@
     <t>Het type distributie. Opties zijn 'deterministic', 'log_normal', 'normal', 'cdf_curve' en 'anders'. De laatste geldt enkel voor de buitenwaterstand.</t>
   </si>
   <si>
-    <t>distributie_type</t>
-  </si>
-  <si>
     <t>Beschrijving</t>
   </si>
   <si>
@@ -252,6 +249,18 @@
   </si>
   <si>
     <t>maximum</t>
+  </si>
+  <si>
+    <t>Vak naam</t>
+  </si>
+  <si>
+    <t>vak_naam</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optioneel invullen. Wordt niet geïmporteerd. </t>
+  </si>
+  <si>
+    <t>distribution_type</t>
   </si>
 </sst>
 </file>
@@ -770,46 +779,46 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DAEDF215-1BC2-44F5-8521-4305F21BD459}">
   <dimension ref="A1:E6"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.28515625" style="14" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="60.5703125" style="14" customWidth="1"/>
-    <col min="3" max="3" width="52.7109375" style="14" customWidth="1"/>
-    <col min="4" max="4" width="25.140625" style="14" customWidth="1"/>
-    <col min="5" max="5" width="26.42578125" style="14" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="8.85546875" style="14"/>
+    <col min="1" max="1" width="23.33203125" style="14" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="60.5546875" style="14" customWidth="1"/>
+    <col min="3" max="3" width="52.6640625" style="14" customWidth="1"/>
+    <col min="4" max="4" width="25.109375" style="14" customWidth="1"/>
+    <col min="5" max="5" width="26.44140625" style="14" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="8.88671875" style="14"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="26.25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="25.8" x14ac:dyDescent="0.3">
       <c r="A1" s="20" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A3" s="12" t="s">
         <v>12</v>
       </c>
       <c r="B3" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="D3" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="C3" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="D3" s="12" t="s">
+      <c r="E3" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="E3" s="12" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="13"/>
       <c r="B4" s="13"/>
       <c r="C4" s="13"/>
       <c r="D4" s="13"/>
       <c r="E4" s="13"/>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="13" t="s">
         <v>9</v>
       </c>
@@ -826,15 +835,15 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="15" t="s">
         <v>0</v>
       </c>
       <c r="B6" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" s="15" t="s">
         <v>26</v>
-      </c>
-      <c r="C6" s="15" t="s">
-        <v>27</v>
       </c>
       <c r="D6" s="15" t="s">
         <v>13</v>
@@ -856,129 +865,140 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9313D639-575E-4463-A991-9636CAC84E2D}">
-  <dimension ref="A1:C21"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:D21"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.28515625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="45.5703125" style="2" customWidth="1"/>
-    <col min="3" max="3" width="13" style="2" customWidth="1"/>
-    <col min="4" max="16384" width="8.85546875" style="2"/>
+    <col min="1" max="1" width="13.33203125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="25.77734375" style="2" customWidth="1"/>
+    <col min="3" max="3" width="45.5546875" style="2" customWidth="1"/>
+    <col min="4" max="4" width="13" style="2" customWidth="1"/>
+    <col min="5" max="16384" width="8.88671875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>8</v>
       </c>
       <c r="B2" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="D2" s="4" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:3" s="6" customFormat="1" ht="12" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" s="6" customFormat="1" ht="12" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>2</v>
       </c>
       <c r="B3" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="D3" s="5" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C4" s="7"/>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C5" s="7"/>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C6" s="7"/>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C7" s="7"/>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C8" s="7"/>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C9" s="7"/>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C10" s="7"/>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C11" s="7"/>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C12" s="7"/>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C13" s="7"/>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C14" s="7"/>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C15" s="7"/>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C16" s="7"/>
-    </row>
-    <row r="17" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C17" s="7"/>
-    </row>
-    <row r="18" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C18" s="7"/>
-    </row>
-    <row r="19" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C19" s="7"/>
-    </row>
-    <row r="20" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C20" s="7"/>
-    </row>
-    <row r="21" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C21" s="7"/>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D4" s="7"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D5" s="7"/>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D6" s="7"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D7" s="7"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D8" s="7"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D9" s="7"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D10" s="7"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D11" s="7"/>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D12" s="7"/>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D13" s="7"/>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D14" s="7"/>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D15" s="7"/>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D16" s="7"/>
+    </row>
+    <row r="17" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D17" s="7"/>
+    </row>
+    <row r="18" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D18" s="7"/>
+    </row>
+    <row r="19" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D19" s="7"/>
+    </row>
+    <row r="20" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D20" s="7"/>
+    </row>
+    <row r="21" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D21" s="7"/>
     </row>
   </sheetData>
-  <autoFilter ref="A3:C3" xr:uid="{9313D639-575E-4463-A991-9636CAC84E2D}"/>
+  <autoFilter ref="A3:D3" xr:uid="{9313D639-575E-4463-A991-9636CAC84E2D}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E90D4119-5ABA-4602-81BD-BF6C31F178E4}">
   <dimension ref="A1:M4"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="22.85546875" style="11" customWidth="1"/>
-    <col min="3" max="3" width="18.42578125" style="11" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="27.140625" style="11" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.7109375" style="11" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="21.5703125" style="11" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.85546875" style="11" customWidth="1"/>
-    <col min="8" max="8" width="12.28515625" style="11" customWidth="1"/>
-    <col min="9" max="9" width="8.42578125" style="11" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.85546875" style="11" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="16.7109375" style="11" customWidth="1"/>
-    <col min="12" max="12" width="38.85546875" style="11" customWidth="1"/>
+    <col min="1" max="2" width="22.88671875" style="11" customWidth="1"/>
+    <col min="3" max="3" width="18.44140625" style="11" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="27.109375" style="11" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.6640625" style="11" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21.5546875" style="11" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.88671875" style="11" customWidth="1"/>
+    <col min="8" max="8" width="12.33203125" style="11" customWidth="1"/>
+    <col min="9" max="9" width="8.44140625" style="11" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.88671875" style="11" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16.6640625" style="11" customWidth="1"/>
+    <col min="12" max="12" width="38.88671875" style="11" customWidth="1"/>
     <col min="13" max="13" width="66" style="11" customWidth="1"/>
-    <col min="14" max="16384" width="8.85546875" style="11"/>
+    <col min="14" max="16384" width="8.88671875" style="11"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="8" t="s">
         <v>12</v>
       </c>
@@ -990,30 +1010,30 @@
         <v>15</v>
       </c>
       <c r="E1" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="F1" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="G1" s="8" t="s">
+      <c r="H1" s="8" t="s">
         <v>32</v>
-      </c>
-      <c r="H1" s="8" t="s">
-        <v>33</v>
       </c>
       <c r="I1" s="8"/>
       <c r="J1" s="8"/>
       <c r="K1" s="8"/>
       <c r="L1" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="M1" s="8" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" ht="126.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" ht="126.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="16" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B2" s="16" t="s">
         <v>17</v>
@@ -1028,7 +1048,7 @@
         <v>20</v>
       </c>
       <c r="F2" s="16" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G2" s="16" t="s">
         <v>16</v>
@@ -1040,11 +1060,11 @@
       <c r="J2" s="16"/>
       <c r="K2" s="16"/>
       <c r="L2" s="16" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="M2" s="16"/>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
         <v>9</v>
       </c>
@@ -1061,25 +1081,25 @@
         <v>9</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G3" s="9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H3" s="9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I3" s="9"/>
       <c r="J3" s="9"/>
       <c r="K3" s="9"/>
       <c r="L3" s="9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="M3" s="9" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" s="10" t="s">
         <v>0</v>
       </c>
@@ -1093,31 +1113,31 @@
         <v>3</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>21</v>
+        <v>71</v>
       </c>
       <c r="F4" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="G4" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="G4" s="10" t="s">
+      <c r="H4" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="H4" s="10" t="s">
+      <c r="I4" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="I4" s="10" t="s">
+      <c r="J4" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="J4" s="10" t="s">
-        <v>68</v>
-      </c>
       <c r="K4" s="10" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="L4" s="10" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="M4" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -1129,47 +1149,47 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A2909D89-B734-46DA-8411-E53B8A7194ED}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.7109375" customWidth="1"/>
+    <col min="1" max="1" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" s="21" t="s">
         <v>58</v>
       </c>
-      <c r="B1" s="21" t="s">
+      <c r="C1" s="21" t="s">
         <v>59</v>
       </c>
-      <c r="C1" s="21" t="s">
+    </row>
+    <row r="2" spans="1:3" ht="69" x14ac:dyDescent="0.3">
+      <c r="A2" s="22" t="s">
         <v>60</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" ht="63.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="22" t="s">
-        <v>61</v>
       </c>
       <c r="B2" s="22"/>
       <c r="C2" s="22"/>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="23" t="s">
         <v>9</v>
       </c>
       <c r="B3" s="23" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C3" s="23" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="24" t="s">
+        <v>61</v>
+      </c>
+      <c r="B4" s="24" t="s">
         <v>62</v>
-      </c>
-      <c r="B4" s="24" t="s">
-        <v>63</v>
       </c>
       <c r="C4" s="24" t="s">
         <v>5</v>
@@ -1183,131 +1203,131 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BEE6525A-680B-4461-9F3B-3E1CE43163B1}">
   <dimension ref="A1:G21"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13" style="2" customWidth="1"/>
-    <col min="2" max="2" width="72.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="44.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.85546875" style="2"/>
-    <col min="5" max="6" width="10.7109375" style="2" customWidth="1"/>
+    <col min="2" max="2" width="72.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="44.109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.88671875" style="2"/>
+    <col min="5" max="6" width="10.6640625" style="2" customWidth="1"/>
     <col min="7" max="7" width="35" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="8.85546875" style="2"/>
+    <col min="8" max="16384" width="8.88671875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="B1" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="17" t="s">
-        <v>41</v>
-      </c>
       <c r="C1" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="D1" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="E1" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="F1" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="G1" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="D1" s="17" t="s">
-        <v>49</v>
-      </c>
-      <c r="E1" s="17" t="s">
-        <v>50</v>
-      </c>
-      <c r="F1" s="17" t="s">
-        <v>53</v>
-      </c>
-      <c r="G1" s="17" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:7" ht="48" x14ac:dyDescent="0.3">
       <c r="A2" s="19" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B2" s="19"/>
       <c r="C2" s="18"/>
       <c r="D2" s="18"/>
       <c r="E2" s="19" t="s">
+        <v>50</v>
+      </c>
+      <c r="F2" s="19" t="s">
+        <v>53</v>
+      </c>
+      <c r="G2" s="18"/>
+    </row>
+    <row r="3" spans="1:7" s="6" customFormat="1" ht="12" x14ac:dyDescent="0.3">
+      <c r="A3" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="B3" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="C3" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="D3" s="18" t="s">
+        <v>47</v>
+      </c>
+      <c r="E3" s="18" t="s">
         <v>51</v>
       </c>
-      <c r="F2" s="19" t="s">
+      <c r="F3" s="18" t="s">
         <v>54</v>
       </c>
-      <c r="G2" s="18"/>
-    </row>
-    <row r="3" spans="1:7" s="6" customFormat="1" ht="12" x14ac:dyDescent="0.25">
-      <c r="A3" s="18" t="s">
-        <v>43</v>
-      </c>
-      <c r="B3" s="18" t="s">
-        <v>42</v>
-      </c>
-      <c r="C3" s="18" t="s">
-        <v>47</v>
-      </c>
-      <c r="D3" s="18" t="s">
-        <v>48</v>
-      </c>
-      <c r="E3" s="18" t="s">
-        <v>52</v>
-      </c>
-      <c r="F3" s="18" t="s">
+      <c r="G3" s="18" t="s">
         <v>55</v>
       </c>
-      <c r="G3" s="18" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="C4" s="7"/>
       <c r="G4" s="7"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="C5" s="7"/>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="C6" s="7"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="C7" s="7"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="C8" s="7"/>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="C9" s="7"/>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="C10" s="7"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="C11" s="7"/>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="C12" s="7"/>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="C13" s="7"/>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="C14" s="7"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="C15" s="7"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="C16" s="7"/>
     </row>
-    <row r="17" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C17" s="7"/>
     </row>
-    <row r="18" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C18" s="7"/>
     </row>
-    <row r="19" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C19" s="7"/>
     </row>
-    <row r="20" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C20" s="7"/>
     </row>
-    <row r="21" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C21" s="7"/>
     </row>
   </sheetData>

</xml_diff>